<commit_message>
feat(F-NAR-019): ATOM-DIF.PAR.002-07 Nino laisse le temps à Aniss
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.PAR.002-07.xlsx
+++ b/stories/arbres/ATOM-DIF.PAR.002-07.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le coquillage de Victorino</t>
+          <t>Nino laisse le temps à Aniss</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>salon, coquillage</t>
+          <t>salon, lampe, table, boîte, fenêtre, rideau, coquillage beige, ligne rose</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Aniss, Victorino, maman, papa</t>
+          <t>Nino, Aniss, papa, maman</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Papa pose un coquillage. Victorino veut raconter. Aniss attend. Victorino dit : un escargot. Ils écoutent encore le silence du coquillage.</t>
+          <t>La lampe fait un rond chaud. Sur le bord, un éclat de coquillage luit. Nino veut raconter, maintenant, ce qu'il y a dedans. Aniss dit j'ai vu, cherche le mot. Nino connaît, ouvre la bouche maintenant, la referme, attend. Escargot. Merci vécu. Deuxième ruse : l'oreille, la mer. Un éclat de coquillage tient sur le bord.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Un coquillage beige repose sur la table basse. Il est un peu rugueux sous le doigt. Une ligne rose tourne à l'intérieur. La fenêtre est déjà bleue. Une couverture en laine attend sur le canapé. Le canapé craque un peu. Je pose le coquillage ici. Il vient de la boîte. On parle tout doux, d'accord ? D'accord, maman. En ce moment, Aniss s'assoit par terre. Le tapis pique un tout petit peu. Tu veux toucher le coquillage ? Oui. Il est froid. On le pose tout doux, d'accord ? D'accord. Victorino s'assoit aussi. Il veut raconter. J'ai vu... Il cherche le mot. Aniss connaît le mot. Il ouvre la bouche. On peut laisser le temps. On attend la fin de la phrase. Aniss referme la bouche. Il pose ses mains. Il attend. J'ai vu un escargot. Dans le coquillage ? Oui. Bravo, Aniss. Tu as laissé le temps. Papa écoute aussi. Il est... Victorino cherche encore. Aniss attend encore. Le temps est doux. Il est petit. Tu as fini ta phrase, Victorino. Aniss, tu as écouté ? Oui, maman. Aniss approche l'oreille. Le coquillage est calme. Tu entends la mer ? Un petit bruit. On laisse le temps. Après, il... Victorino cherche encore. Aniss attend. La couverture sent la laine. Après, il rentre. Dans sa maison. Vous avez parlé l'un après l'autre. Aniss, tu as attendu la fin ? Oui, papa. Victorino finit sa phrase. Aniss attend encore. On touche encore le coquillage ? Oui. Tout doux. Tu comptes les lignes roses ? Une. Deux. Trois. Moi, je... Aniss attend. Moi, je compte aussi. Vous avez laissé le temps.</t>
+          <t>La lampe fait un rond chaud. Il est chaud, papa. Tu le vois, le rond, Nino ? Oui, papa. Le rond pose sur la table. La table est claire, ce soir. Oui, maman. La fenêtre est bleue, dehors. Tu vois le bleu, Nino ? Oui, il est bleu. Papa ouvre une petite boîte. La boîte sent le bois sec. Ça sent le bois, papa. Tu entends le couvercle ? Oui, il claque. Un coquillage beige sort. Il est un peu rugueux. Il pique un peu, maman. Sous le doigt ? Oui. Une ligne rose tourne dedans. Elle est rose. Tu la vois, la ligne ? Oui, papa. Sur le bord, un éclat de coquillage luit. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. La lampe le touche. Nino pose la paume dessus. Le coquillage est froid. Il est froid. Tu le tiens, Nino ? Oui. En ce moment, Nino le lève. Je veux raconter, maintenant ! Ce qu'il y a dedans. Tout de suite ? Oui, papa. Aniss arrive près de la table. Il regarde le coquillage. J'ai vu. Aniss cherche le mot. Sa bouche reste ouverte. Nino connaît le mot. Il ouvre la bouche, maintenant. Le mot pousse, tout près. Ses lèvres bougent. Oh. Le sourire de Nino disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'attente se heurtent. Il referme la bouche. Il pose ses mains. Personne ne dit le mot. Papa s'accroupit à la même hauteur. Tu vois Aniss, Nino ? Oui, papa. Tes mains sont froides, Nino ? Un peu, maman. L'éclat de coquillage tremble, puis tient.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Un coquillage beige repose sur la table basse. Il est un peu rugueux sous le doigt. Une ligne rose tourne à l'intérieur. La fenêtre est déjà bleue. Une couverture en laine attend sur le canapé. Le canapé craque un peu. Je pose le coquillage ici. Il vient de la boîte. On parle tout doux, d'accord ? D'accord, maman. En ce moment, Aniss s'assoit par terre. Le tapis pique un tout petit peu. Tu veux toucher le coquillage ? Oui. Il est froid. On le pose tout doux, d'accord ? D'accord. Victorino s'assoit aussi. Il veut raconter. J'ai vu... Il cherche le mot. Aniss connaît le mot. Il ouvre la bouche. On peut laisser le temps. On attend la fin de la phrase. Aniss referme la bouche. Il pose ses mains. Il attend. J'ai vu un escargot. Dans le coquillage ? Oui. Bravo, Aniss. Tu as laissé le temps. Papa écoute aussi. Il est... Victorino cherche encore. Aniss attend encore. Le temps est doux. Il est petit. Tu as fini ta phrase, Victorino. Aniss, tu as écouté ? Oui, maman. Aniss approche l'oreille. Le coquillage est calme. Tu entends la mer ? Un petit bruit. On laisse le temps. Après, il... Victorino cherche encore. Aniss attend. La couverture sent la laine. Après, il rentre. Dans sa maison. Vous avez parlé l'un après l'autre. Aniss, tu as attendu la fin ? Oui, papa. Victorino finit sa phrase. Aniss attend encore. On touche encore le coquillage ? Oui. Tout doux. Tu comptes les lignes roses ? Une. Deux. Trois. Moi, je... Aniss attend. Moi, je compte aussi. Vous avez laissé le temps.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La lampe fait un rond chaud. Il est chaud, papa. Tu le vois, le rond, Nino ? Oui, papa. Le rond pose sur la table. La table est claire, ce soir. Oui, maman. La fenêtre est bleue, dehors. Tu vois le bleu, Nino ? Oui, il est bleu. Papa ouvre une petite boîte. La boîte sent le bois sec. Ça sent le bois, papa. Tu entends le couvercle ? Oui, il claque. Un coquillage beige sort. Il est un peu rugueux. Il pique un peu, maman. Sous le doigt ? Oui. Une ligne rose tourne dedans. Elle est rose. Tu la vois, la ligne ? Oui, papa. Sur le bord, un &lt;emphasis level="moderate"&gt;éclat de coquillage&lt;/emphasis&gt; luit. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. La lampe le touche. Nino pose la paume dessus. Le coquillage est froid. Il est froid. Tu le tiens, Nino ? Oui. En ce moment, Nino le lève. Je veux raconter, maintenant ! Ce qu'il y a dedans. Tout de suite ? Oui, papa. Aniss arrive près de la table. Il regarde le coquillage. J'ai vu. Aniss cherche le mot. Sa bouche reste ouverte. Nino connaît le mot. Il ouvre la bouche, maintenant. Le mot pousse, tout près. Ses lèvres bougent. Oh. Le sourire de Nino disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'attente se heurtent. Il referme la bouche. Il pose ses mains. Personne ne dit le mot. Papa s'accroupit à la même hauteur. Tu vois Aniss, Nino ? Oui, papa. Tes mains sont froides, Nino ? Un peu, maman. L'éclat de coquillage tremble, puis tient.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Didier est dans le salon. Papa pose un coquillage. Jules veut raconter. Jules dit : j'ai vu.. Puis il cherche le mot. Didier connaît le mot. Il ouvre la bouche. Maman dit : on peut &lt;emphasis&gt;laisser&lt;/emphasis&gt; le temps. On n'achève pas à sa place. Didier attend la fin de la phrase. Il laisse le temps. Jules dit : j'ai vu un escargot. Didier sourit. Il a su laisser le temps. Papa écoute aussi. Jules finit sa phrase. Didier attend encore. Le temps est doux.&lt;/slow&gt; [pause]</t>
+          <t>La lampe fait un rond chaud. Il est chaud, papa. Tu le vois, le rond, Nino ? Oui, papa. Le rond pose sur la table. La table est claire, ce soir. Oui, maman. La fenêtre est bleue, dehors. Tu vois le bleu, Nino ? Oui, il est bleu. Papa ouvre une petite boîte. La boîte sent le bois sec. Ça sent le bois, papa. Tu entends le couvercle ? Oui, il claque. Un coquillage beige sort. Il est un peu rugueux. Il pique un peu, maman. Sous le doigt ? Oui. Une ligne rose tourne dedans. Elle est rose. Tu la vois, la ligne ? Oui, papa. Sur le bord, un &lt;emphasis&gt;éclat de coquillage&lt;/emphasis&gt; luit. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. La lampe le touche. Nino pose la paume dessus. Le coquillage est froid. Il est froid. Tu le tiens, Nino ? Oui. En ce moment, Nino le lève. Je veux raconter, maintenant ! Ce qu'il y a dedans. Tout de suite ? Oui, papa. Aniss arrive près de la table. Il regarde le coquillage. J'ai vu. Aniss cherche le mot. Sa bouche reste ouverte. Nino connaît le mot. Il ouvre la bouche, maintenant. Le mot pousse, tout près. Ses lèvres bougent. Oh. Le sourire de Nino disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'attente se heurtent. Il referme la bouche. Il pose ses mains. Personne ne dit le mot. Papa s'accroupit à la même hauteur. Tu vois Aniss, Nino ? Oui, papa. Tes mains sont froides, Nino ? Un peu, maman. L'éclat de coquillage tremble, puis tient. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,18 +1241,18 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.28</v>
+        <v>1.22</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>laisser</t>
+          <t>éclat de coquillage</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>560</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>300</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1319,80 +1319,76 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis retenue; intensite=2; destinataire=enfant; sous_texte=il_veut_raconter_maintenant; tempo=posé puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Un coquillage beige repose sur la table basse.
-narrateur|Il est un peu rugueux sous le doigt.
-narrateur|Une ligne rose tourne à l'intérieur.
-narrateur|La fenêtre est déjà bleue.
-narrateur|Une couverture en laine attend sur le canapé.
-narrateur|Le canapé craque un peu.
-papa|Je pose le coquillage ici.
-papa|Il vient de la boîte.
-maman|On parle tout doux, d'accord ?
-enfant-m|D'accord, maman.
-narrateur|En ce moment, Aniss s'assoit par terre.
-narrateur|Le tapis pique un tout petit peu.
-papa|Tu veux toucher le coquillage ?
+          <t>narrateur|La lampe fait un rond chaud.
+enfant-m|Il est chaud, papa.
+papa|Tu le vois, le rond, Nino ?
+enfant-m|Oui, papa.
+narrateur|Le rond pose sur la table.
+maman|La table est claire, ce soir.
+enfant-m|Oui, maman.
+narrateur|La fenêtre est bleue, dehors.
+papa|Tu vois le bleu, Nino ?
+enfant-m|Oui, il est bleu.
+narrateur|Papa ouvre une petite boîte.
+narrateur|La boîte sent le bois sec.
+enfant-m|Ça sent le bois, papa.
+papa|Tu entends le couvercle ?
+enfant-m|Oui, il claque.
+narrateur|Un coquillage beige sort.
+narrateur|Il est un peu rugueux.
+enfant-m|Il pique un peu, maman.
+maman|Sous le doigt ?
 enfant-m|Oui.
+narrateur|Une ligne rose tourne dedans.
+enfant-m|Elle est rose.
+papa|Tu la vois, la ligne ?
+enfant-m|Oui, papa.
+narrateur|Sur le bord, un éclat de coquillage luit.
+enfant-m|Il brille, maman.
+maman|Tu le vois, le petit point ?
+enfant-m|Oui, un petit point.
+papa|La lampe le touche.
+narrateur|Nino pose la paume dessus.
+narrateur|Le coquillage est froid.
 enfant-m|Il est froid.
-maman|On le pose tout doux, d'accord ?
-enfant-m|D'accord.
-narrateur|Victorino s'assoit aussi.
-narrateur|Il veut raconter.
-copain|J'ai vu...
-narrateur|Il cherche le mot.
-narrateur|Aniss connaît le mot.
-narrateur|Il ouvre la bouche.
-maman|On peut laisser le temps.
-maman|On attend la fin de la phrase.
-narrateur|Aniss referme la bouche.
+maman|Tu le tiens, Nino ?
+enfant-m|Oui.
+narrateur|En ce moment, Nino le lève.
+enfant-m|Je veux raconter, maintenant !
+enfant-m|Ce qu'il y a dedans.
+papa|Tout de suite ?
+enfant-m|Oui, papa.
+narrateur|Aniss arrive près de la table.
+narrateur|Il regarde le coquillage.
+copain|J'ai vu.
+narrateur|Aniss cherche le mot.
+narrateur|Sa bouche reste ouverte.
+narrateur|Nino connaît le mot.
+narrateur|Il ouvre la bouche, maintenant.
+narrateur|Le mot pousse, tout près.
+narrateur|Ses lèvres bougent.
+enfant-m|Oh.
+narrateur|Le sourire de Nino disparaît.
+narrateur|Dans sa poitrine, ça se bouscule.
+narrateur|L'envie et l'attente se heurtent.
+narrateur|Il referme la bouche.
 narrateur|Il pose ses mains.
-narrateur|Il attend.
-copain|J'ai vu un escargot.
-enfant-m|Dans le coquillage ?
-copain|Oui.
-papa|Bravo, Aniss.
-papa|Tu as laissé le temps.
-narrateur|Papa écoute aussi.
-copain|Il est...
-narrateur|Victorino cherche encore.
-narrateur|Aniss attend encore.
-narrateur|Le temps est doux.
-copain|Il est petit.
-maman|Tu as fini ta phrase, Victorino.
-maman|Aniss, tu as écouté ?
-enfant-m|Oui, maman.
-narrateur|Aniss approche l'oreille.
-narrateur|Le coquillage est calme.
-papa|Tu entends la mer ?
-enfant-m|Un petit bruit.
-maman|On laisse le temps.
-copain|Après, il...
-narrateur|Victorino cherche encore.
-narrateur|Aniss attend.
-narrateur|La couverture sent la laine.
-copain|Après, il rentre.
-enfant-m|Dans sa maison.
-papa|Vous avez parlé l'un après l'autre.
-papa|Aniss, tu as attendu la fin ?
+narrateur|Personne ne dit le mot.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu vois Aniss, Nino ?
 enfant-m|Oui, papa.
-narrateur|Victorino finit sa phrase.
-narrateur|Aniss attend encore.
-maman|On touche encore le coquillage ?
-enfant-m|Oui.
-enfant-m|Tout doux.
-papa|Tu comptes les lignes roses ?
-enfant-m|Une.
-enfant-m|Deux.
-enfant-m|Trois.
-copain|Moi, je...
-narrateur|Aniss attend.
-copain|Moi, je compte aussi.
-maman|Vous avez laissé le temps.</t>
+maman|Tes mains sont froides, Nino ?
+enfant-m|Un peu, maman.
+narrateur|L'éclat de coquillage tremble, puis tient.</t>
         </is>
       </c>
     </row>
@@ -1419,17 +1415,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Victorino cherche un mot. Que fait Aniss ?</t>
+          <t>Aniss cherche un mot. Que fait Nino ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Victorino cherche un mot. Que fait Aniss ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Aniss cherche un &lt;emphasis level="moderate"&gt;mot&lt;/emphasis&gt;. Que fait Nino ?&lt;/prosody&gt;&lt;break time="780ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Jules cherche un mot. Que fait Didier ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Aniss cherche un &lt;emphasis&gt;mot&lt;/emphasis&gt;. Que fait Nino ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1454,7 +1450,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>On n'achève pas à sa place. Que fait Didier ?</t>
+          <t>On n'achève pas à sa place. Que fait Nino ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1492,7 +1488,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1503,7 +1499,7 @@
         <v>0.8</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.4</v>
+        <v>1.36</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1518,34 +1514,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>mot</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>780</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>360</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.3</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1560,7 +1560,7 @@
         <v>0.8</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1570,13 +1570,13 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=aniss_cherche_un_mot_que_fait_nino; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Victorino cherche un mot.
-narrateur|Que fait Aniss ?</t>
+          <t>narrateur|Aniss cherche un mot.
+narrateur|Que fait Nino ?</t>
         </is>
       </c>
     </row>
@@ -1603,17 +1603,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Aniss a su laisser le temps. Victorino a fini sa phrase. On laisse le temps. Bravo, Aniss. J'ai attendu.</t>
+          <t>Nino garde la bouche fermée. Aniss cherche, un instant. J'ai vu un escargot. Dans le coquillage ? Oui. Merci, Nino. Papa a vu les deux, près de la table. La ligne rose est là, Aniss ? Oui. Elle tourne. Nino approche l'oreille. Le coquillage est calme. Tu entends un bruit, Nino ? Un petit bruit. Aniss, tu entends aussi ? Un peu. Le ventre de Nino se desserre. Les épaules se relèvent un peu. Il est petit. Oui, petit. On reste près de la table ? Oui. Tes mains sont au chaud ? Un peu, maman. Ils posent le coquillage. La lampe tient le rond. Il brille. Tu le vois, le bord ? Oui, papa.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Aniss a su laisser le temps. Victorino a fini sa phrase. On laisse le temps. Bravo, Aniss. J'ai attendu.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino garde la bouche fermée. Aniss cherche, un instant. J'ai vu un &lt;emphasis level="moderate"&gt;escargot&lt;/emphasis&gt;. Dans le coquillage ? Oui. Merci, Nino. Papa a vu les deux, près de la table. La ligne rose est là, Aniss ? Oui. Elle tourne. Nino approche l'oreille. Le coquillage est calme. Tu entends un bruit, Nino ? Un petit bruit. Aniss, tu entends aussi ? Un peu. Le ventre de Nino se desserre. Les épaules se relèvent un peu. Il est petit. Oui, petit. On reste près de la table ? Oui. Tes mains sont au chaud ? Un peu, maman. Ils posent le coquillage. La lampe tient le rond. Il brille. Tu le vois, le bord ? Oui, papa.&lt;/prosody&gt;&lt;break time="620ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Didier a su &lt;emphasis&gt;laisser&lt;/emphasis&gt; le temps. Jules a fini sa phrase. Papa et maman ont vu.&lt;/slow&gt; [pause]</t>
+          <t>Nino garde la bouche fermée. Aniss cherche, un instant. J'ai vu un &lt;emphasis&gt;escargot&lt;/emphasis&gt;. Dans le coquillage ? Oui. Merci, Nino. Papa a vu les deux, près de la table. La ligne rose est là, Aniss ? Oui. Elle tourne. Nino approche l'oreille. Le coquillage est calme. Tu entends un bruit, Nino ? Un petit bruit. Aniss, tu entends aussi ? Un peu. Le ventre de Nino se desserre. Les épaules se relèvent un peu. Il est petit. Oui, petit. On reste près de la table ? Oui. Tes mains sont au chaud ? Un peu, maman. Ils posent le coquillage. La lampe tient le rond. Il brille. Tu le vois, le bord ? Oui, papa. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1660,18 +1660,18 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.28</v>
+        <v>1.24</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1694,30 +1694,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>laisser</t>
+          <t>escargot</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>620</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>310</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.33</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1726,10 +1726,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1738,20 +1738,44 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_referme_la_bouche_aniss_trouve; tempo=posé; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Aniss a su laisser le temps.
-narrateur|Victorino a fini sa phrase.
-maman|On laisse le temps.
-papa|Bravo, Aniss.
-enfant-m|J'ai attendu.</t>
+          <t>narrateur|Nino garde la bouche fermée.
+narrateur|Aniss cherche, un instant.
+copain|J'ai vu un escargot.
+enfant-m|Dans le coquillage ?
+copain|Oui.
+papa|Merci, Nino.
+narrateur|Papa a vu les deux, près de la table.
+maman|La ligne rose est là, Aniss ?
+copain|Oui.
+enfant-m|Elle tourne.
+narrateur|Nino approche l'oreille.
+narrateur|Le coquillage est calme.
+papa|Tu entends un bruit, Nino ?
+enfant-m|Un petit bruit.
+maman|Aniss, tu entends aussi ?
+copain|Un peu.
+narrateur|Le ventre de Nino se desserre.
+narrateur|Les épaules se relèvent un peu.
+enfant-m|Il est petit.
+copain|Oui, petit.
+papa|On reste près de la table ?
+enfant-m|Oui.
+maman|Tes mains sont au chaud ?
+enfant-m|Un peu, maman.
+narrateur|Ils posent le coquillage.
+narrateur|La lampe tient le rond.
+enfant-m|Il brille.
+papa|Tu le vois, le bord ?
+enfant-m|Oui, papa.</t>
         </is>
       </c>
     </row>
@@ -1778,17 +1802,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Aniss pose le coquillage. Tout doux, sur la table. Il est à sa place. Oui. Merci, Aniss. On peut... Victorino cherche. Aniss attend. On peut le recouvrir. Avec la couverture ? D'accord. Tu as encore laissé le temps. La couverture sent la laine. La fenêtre est encore bleue.</t>
+          <t>Maman approche le coquillage. Elle le tend vers Aniss. J'écoute, maintenant ! Aniss le pose contre l'oreille. J'entends. Aniss cherche le mot. Sa bouche reste ouverte. Nino connaît le mot. Il ouvre la bouche, trop vite. Le mot pousse, tout près. Oh. Nino referme la bouche. Il pose ses mains. Personne ne dit la suite. Sur le bord, un éclat de coquillage luit. Là, sur le bord. Tu entends, Aniss ? Aniss ne dit rien. Il souffle, puis écoute. La mer. Dans le coquillage ? Oui. On range la boîte ? Oui, papa. La boîte sent le bois sec. Le coquillage glisse dedans. Il est à sa place. Le couvercle, Aniss ? Oui. La lampe est calme, Nino ? Oui, papa. Un rond reste sur la table. Il allume le bord.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Aniss pose le coquillage. Tout doux, sur la table. Il est à sa place. Oui. Merci, Aniss. On peut... Victorino cherche. Aniss attend. On peut le recouvrir. Avec la couverture ? D'accord. Tu as encore laissé le temps. La couverture sent la laine. La fenêtre est encore bleue.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Maman approche le coquillage. Elle le tend vers Aniss. J'écoute, maintenant ! Aniss le pose contre l'oreille. J'entends. Aniss cherche le mot. Sa bouche reste ouverte. Nino connaît le mot. Il ouvre la bouche, trop vite. Le mot pousse, tout près. Oh. Nino referme la bouche. Il pose ses mains. Personne ne dit la suite. Sur le bord, un &lt;emphasis level="moderate"&gt;éclat de coquillage&lt;/emphasis&gt; luit. Là, sur le bord. Tu entends, Aniss ? Aniss ne dit rien. Il souffle, puis écoute. La mer. Dans le coquillage ? Oui. On range la boîte ? Oui, papa. La boîte sent le bois sec. Le coquillage glisse dedans. Il est à sa place. Le couvercle, Aniss ? Oui. La lampe est calme, Nino ? Oui, papa. Un rond reste sur la table. Il allume le bord.&lt;/prosody&gt;&lt;break time="480ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Didier pose le coquillage. Maman sourit.&lt;/slow&gt; [pause]</t>
+          <t>Maman approche le coquillage. Elle le tend vers Aniss. J'écoute, maintenant ! Aniss le pose contre l'oreille. J'entends. Aniss cherche le mot. Sa bouche reste ouverte. Nino connaît le mot. Il ouvre la bouche, trop vite. Le mot pousse, tout près. Oh. Nino referme la bouche. Il pose ses mains. Personne ne dit la suite. Sur le bord, un &lt;emphasis&gt;éclat de coquillage&lt;/emphasis&gt; luit. Là, sur le bord. Tu entends, Aniss ? Aniss ne dit rien. Il souffle, puis écoute. La mer. Dans le coquillage ? Oui. On range la boîte ? Oui, papa. La boîte sent le bois sec. Le coquillage glisse dedans. Il est à sa place. Le couvercle, Aniss ? Oui. La lampe est calme, Nino ? Oui, papa. Un rond reste sur la table. Il allume le bord. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1835,18 +1859,18 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.28</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1867,28 +1891,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de coquillage</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>480</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>280</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1897,10 +1925,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1909,25 +1937,48 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=l_oreille_la_mer_il_referme_encore; tempo=un peu vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Aniss pose le coquillage.
-papa|Tout doux, sur la table.
+          <t>narrateur|Maman approche le coquillage.
+narrateur|Elle le tend vers Aniss.
+enfant-m|J'écoute, maintenant !
+narrateur|Aniss le pose contre l'oreille.
+copain|J'entends.
+narrateur|Aniss cherche le mot.
+narrateur|Sa bouche reste ouverte.
+narrateur|Nino connaît le mot.
+narrateur|Il ouvre la bouche, trop vite.
+narrateur|Le mot pousse, tout près.
+enfant-m|Oh.
+narrateur|Nino referme la bouche.
+narrateur|Il pose ses mains.
+narrateur|Personne ne dit la suite.
+narrateur|Sur le bord, un éclat de coquillage luit.
+enfant-m|Là, sur le bord.
+enfant-m|Tu entends, Aniss ?
+narrateur|Aniss ne dit rien.
+narrateur|Il souffle, puis écoute.
+copain|La mer.
+enfant-m|Dans le coquillage ?
+copain|Oui.
+papa|On range la boîte ?
+enfant-m|Oui, papa.
+narrateur|La boîte sent le bois sec.
+narrateur|Le coquillage glisse dedans.
 enfant-m|Il est à sa place.
-maman|Oui.
-maman|Merci, Aniss.
-copain|On peut...
-narrateur|Victorino cherche.
-narrateur|Aniss attend.
-copain|On peut le recouvrir.
-maman|Avec la couverture ?
-maman|D'accord.
-papa|Tu as encore laissé le temps.
-narrateur|La couverture sent la laine.
-narrateur|La fenêtre est encore bleue.</t>
+maman|Le couvercle, Aniss ?
+copain|Oui.
+papa|La lampe est calme, Nino ?
+enfant-m|Oui, papa.
+maman|Un rond reste sur la table.
+enfant-m|Il allume le bord.</t>
         </is>
       </c>
     </row>
@@ -1954,17 +2005,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai attendu la fin. Bravo. Le coquillage reste sur la table.</t>
+          <t>Ils restent près de la table. Maman ferme un peu la boîte. Le coquillage est dedans, papa. Tu l'as vu, toi ? Oui, près de la lampe. On est bien, ici. Nino tapote le couvercle du doigt. Il a une trace de bois. Tu la vois, la trace ? Oui, maman. Le coquillage est resté, Nino. Oui, avec Aniss. Le coquillage est resté. Ça sent le bois, un peu tiède. Et la lampe, maman. Oui, dans l'air. La boîte reste sur la table. Un éclat de coquillage tient sur le bord.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai attendu la fin. Bravo. Le coquillage reste sur la table.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de la table. Maman ferme un peu la boîte. Le coquillage est dedans, papa. Tu l'as vu, toi ? Oui, près de la lampe. On est bien, ici. Nino tapote le couvercle du doigt. Il a une trace de bois. Tu la vois, la trace ? Oui, maman. Le coquillage est resté, Nino. Oui, avec Aniss. Le coquillage est resté. Ça sent le bois, un peu tiède. Et la lampe, maman. Oui, dans l'air. La boîte reste sur la table. Un &lt;emphasis level="moderate"&gt;éclat de coquillage&lt;/emphasis&gt; tient sur le bord.&lt;/prosody&gt;&lt;break time="980ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de la table. Maman ferme un peu la boîte. Le coquillage est dedans, papa. Tu l'as vu, toi ? Oui, près de la lampe. On est bien, ici. Nino tapote le couvercle du doigt. Il a une trace de bois. Tu la vois, la trace ? Oui, maman. Le coquillage est resté, Nino. Oui, avec Aniss. Le coquillage est resté. Ça sent le bois, un peu tiède. Et la lampe, maman. Oui, dans l'air. La boîte reste sur la table. Un &lt;emphasis&gt;éclat de coquillage&lt;/emphasis&gt; tient sur le bord.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2011,7 +2062,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2019,7 +2070,7 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AB6" s="2" t="n">
         <v>1.36</v>
@@ -2031,12 +2082,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2045,14 +2096,18 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de coquillage</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>980</v>
       </c>
       <c r="AK6" s="2" t="n">
         <v>380</v>
@@ -2064,11 +2119,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.29</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2077,26 +2132,45 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_bord; tempo=très posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|J'ai attendu la fin.
-maman|Bravo.
-narrateur|Le coquillage reste sur la table.</t>
+          <t>narrateur|Ils restent près de la table.
+narrateur|Maman ferme un peu la boîte.
+enfant-m|Le coquillage est dedans, papa.
+papa|Tu l'as vu, toi ?
+enfant-m|Oui, près de la lampe.
+maman|On est bien, ici.
+narrateur|Nino tapote le couvercle du doigt.
+enfant-m|Il a une trace de bois.
+maman|Tu la vois, la trace ?
+enfant-m|Oui, maman.
+papa|Le coquillage est resté, Nino.
+enfant-m|Oui, avec Aniss.
+copain|Le coquillage est resté.
+narrateur|Ça sent le bois, un peu tiède.
+enfant-m|Et la lampe, maman.
+maman|Oui, dans l'air.
+narrateur|La boîte reste sur la table.
+narrateur|Un éclat de coquillage tient sur le bord.</t>
         </is>
       </c>
     </row>
@@ -2117,7 +2191,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2181,6 +2255,13 @@
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>